<commit_message>
Polish Benelli shotgun combat, block reload while running, and fix Ctrl facing.
Add ShotgunCqb balance, jittered pellet pattern, scaled visual kick, and combat docs/Excel; interrupt reload/loading on run/sprint; fix single-unit Ctrl HoldToEnd; temporarily disable ready/not-ready root yaw transitions.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Tools/CombatBalanceParameters.xlsx
+++ b/Tools/CombatBalanceParameters.xlsx
@@ -756,6 +756,38 @@
             </numRef>
           </val>
         </ser>
+        <ser>
+          <idx val="18"/>
+          <order val="18"/>
+          <tx>
+            <strRef>
+              <f>'Точность'!T1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Точность'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Точность'!$T$2:$T$12</f>
+            </numRef>
+          </val>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -1418,6 +1450,38 @@
             </numRef>
           </val>
         </ser>
+        <ser>
+          <idx val="18"/>
+          <order val="18"/>
+          <tx>
+            <strRef>
+              <f>'Прицеливание'!T1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Прицеливание'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Прицеливание'!$T$2:$T$12</f>
+            </numRef>
+          </val>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -2077,6 +2141,38 @@
           <val>
             <numRef>
               <f>'Отдача'!$S$2:$S$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="18"/>
+          <order val="18"/>
+          <tx>
+            <strRef>
+              <f>'Отдача'!T1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Отдача'!$A$2:$A$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Отдача'!$T$2:$T$11</f>
             </numRef>
           </val>
         </ser>
@@ -5305,7 +5401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5420,7 +5516,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0, 10, 20 … 100 м — для точности и прицеливания</t>
+          <t>0, 50, 100 … 500 м — для точности и прицеливания</t>
         </is>
       </c>
     </row>
@@ -5461,28 +5557,40 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Benelli M4</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Роль ShotgunCqb: 0–15 лучший, 15–25 сильный, 25–40 рабочий, 40–60 хуже АК, 60+ почти бесполезен. Эффективность дроби = паттерн + falloff, не только лист Точность.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Важно</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Точность и прицеливание читаются из Unity assets. Перезапекание: python Tools/bake_weapon_combat_balance.py</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Важно</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Точность и прицеливание читаются из Unity assets. Перезапекание: python Tools/bake_weapon_combat_balance.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>Обновление</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>python Tools/export_combat_balance_excel.py</t>
         </is>
@@ -5571,7 +5679,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>0.312</v>
@@ -5591,7 +5699,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>0.354</v>
@@ -5611,7 +5719,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0.43</v>
@@ -5631,7 +5739,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>0.539</v>
@@ -5651,7 +5759,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="B8" s="3" t="n">
         <v>0.648</v>
@@ -5671,7 +5779,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>60</v>
+        <v>300</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>0.775</v>
@@ -5691,7 +5799,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>70</v>
+        <v>350</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>0.902</v>
@@ -5711,7 +5819,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>80</v>
+        <v>400</v>
       </c>
       <c r="B11" s="3" t="n">
         <v>1.03</v>
@@ -5731,7 +5839,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>90</v>
+        <v>450</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>1.159</v>
@@ -5751,7 +5859,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="B13" s="3" t="n">
         <v>1.287</v>
@@ -6266,7 +6374,7 @@
         <v>0</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>-0.042</v>
+        <v>-0.04</v>
       </c>
       <c r="P4" s="3" t="n">
         <v>0</v>
@@ -6323,14 +6431,14 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>50–60 м</t>
+          <t>250–300 м</t>
         </is>
       </c>
       <c r="N5" s="3" t="n">
-        <v>-0.003</v>
+        <v>-0.06</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>0.159</v>
+        <v>0.143</v>
       </c>
       <c r="P5" s="3" t="n">
         <v>0</v>
@@ -6394,7 +6502,7 @@
         <v>0</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.02</v>
+        <v>0.015</v>
       </c>
       <c r="P6" s="3" t="n">
         <v>0</v>
@@ -6458,7 +6566,7 @@
         <v>0</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.02</v>
+        <v>0.015</v>
       </c>
       <c r="P7" s="3" t="n">
         <v>0</v>
@@ -6515,14 +6623,14 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>50–50 м</t>
+          <t>250–250 м</t>
         </is>
       </c>
       <c r="N8" s="3" t="n">
-        <v>-0.043</v>
+        <v>-0.124</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.119</v>
+        <v>0.116</v>
       </c>
       <c r="P8" s="3" t="n">
         <v>0</v>
@@ -6579,14 +6687,14 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>50–60 м</t>
+          <t>250–300 м</t>
         </is>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.097</v>
+        <v>0.041</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.081</v>
+        <v>0.075</v>
       </c>
       <c r="P9" s="3" t="n">
         <v>0</v>
@@ -6643,14 +6751,14 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>20–30 м</t>
+          <t>100–150 м</t>
         </is>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.114</v>
+        <v>0.048</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>-0.002</v>
+        <v>-0.004</v>
       </c>
       <c r="P10" s="3" t="n">
         <v>0</v>
@@ -6707,14 +6815,14 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>40–60 м</t>
+          <t>200–300 м</t>
         </is>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.105</v>
+        <v>-0.013</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.094</v>
+        <v>0.1</v>
       </c>
       <c r="P11" s="3" t="n">
         <v>0</v>
@@ -6771,14 +6879,14 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>0–70 м</t>
+          <t>0–350 м</t>
         </is>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.033</v>
+        <v>0.11</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.08</v>
+        <v>0.045</v>
       </c>
       <c r="P12" s="3" t="n">
         <v>0</v>
@@ -6842,7 +6950,7 @@
         <v>0</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.016</v>
+        <v>0.012</v>
       </c>
       <c r="P13" s="3" t="n">
         <v>0</v>
@@ -6906,7 +7014,7 @@
         <v>0</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.016</v>
+        <v>0.012</v>
       </c>
       <c r="P14" s="3" t="n">
         <v>0.103</v>
@@ -6970,7 +7078,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="P15" s="3" t="n">
         <v>0.08</v>
@@ -7034,7 +7142,7 @@
         <v>0</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>-0.026</v>
+        <v>-0.02</v>
       </c>
       <c r="P16" s="3" t="n">
         <v>0.028</v>
@@ -7098,7 +7206,7 @@
         <v>0</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>-0.016</v>
+        <v>-0.012</v>
       </c>
       <c r="P17" s="3" t="n">
         <v>0.048</v>
@@ -7162,7 +7270,7 @@
         <v>0</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>-0.023</v>
+        <v>-0.017</v>
       </c>
       <c r="P18" s="3" t="n">
         <v>0.058</v>
@@ -7219,14 +7327,14 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0–20 м</t>
+          <t>0–0 м</t>
         </is>
       </c>
       <c r="N19" s="3" t="n">
-        <v>0.105</v>
+        <v>0.115</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>0.016</v>
+        <v>0.012</v>
       </c>
       <c r="P19" s="3" t="n">
         <v>0</v>
@@ -7283,7 +7391,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>0–10 м</t>
+          <t>0–0 м</t>
         </is>
       </c>
       <c r="N20" s="3" t="n">
@@ -7354,7 +7462,7 @@
         <v>0</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>-0.029</v>
+        <v>-0.022</v>
       </c>
       <c r="P21" s="3" t="n">
         <v>-0.11</v>
@@ -7418,7 +7526,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>-0.008</v>
+        <v>-0.006</v>
       </c>
       <c r="P22" s="3" t="n">
         <v>0</v>
@@ -7475,14 +7583,14 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0–20 м</t>
+          <t>0–100 м</t>
         </is>
       </c>
       <c r="N23" s="3" t="n">
-        <v>0.025</v>
+        <v>0.126</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>-0.006</v>
+        <v>-0.013</v>
       </c>
       <c r="P23" s="3" t="n">
         <v>0</v>
@@ -7539,14 +7647,14 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>0–10 м</t>
+          <t>0–50 м</t>
         </is>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.025</v>
+        <v>0.126</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>-0.006</v>
+        <v>-0.013</v>
       </c>
       <c r="P24" s="3" t="n">
         <v>0</v>
@@ -7603,14 +7711,14 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>0–20 м</t>
+          <t>0–100 м</t>
         </is>
       </c>
       <c r="N25" s="3" t="n">
-        <v>0.059</v>
+        <v>0.111</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>-0.008999999999999999</v>
+        <v>-0.014</v>
       </c>
       <c r="P25" s="3" t="n">
         <v>0</v>
@@ -7667,14 +7775,14 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>0–20 м</t>
+          <t>0–100 м</t>
         </is>
       </c>
       <c r="N26" s="3" t="n">
-        <v>0.025</v>
+        <v>0.12</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>-0.006</v>
+        <v>-0.013</v>
       </c>
       <c r="P26" s="3" t="n">
         <v>0</v>
@@ -7731,14 +7839,14 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>40–40 м</t>
+          <t>200–200 м</t>
         </is>
       </c>
       <c r="N27" s="3" t="n">
-        <v>0.097</v>
+        <v>-0.12</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>0.054</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="P27" s="3" t="n">
         <v>0</v>
@@ -7795,14 +7903,14 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>60–70 м</t>
+          <t>300–350 м</t>
         </is>
       </c>
       <c r="N28" s="3" t="n">
-        <v>-0.161</v>
+        <v>-0.269</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>0.29</v>
+        <v>0.253</v>
       </c>
       <c r="P28" s="3" t="n">
         <v>0</v>
@@ -7859,14 +7967,14 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>80–100 м</t>
+          <t>400–500 м</t>
         </is>
       </c>
       <c r="N29" s="3" t="n">
-        <v>-0.2</v>
+        <v>-0.315</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>0.337</v>
+        <v>0.3</v>
       </c>
       <c r="P29" s="3" t="n">
         <v>0</v>
@@ -7923,14 +8031,14 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>80–100 м</t>
+          <t>400–500 м</t>
         </is>
       </c>
       <c r="N30" s="3" t="n">
-        <v>-0.247</v>
+        <v>-0.358</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>0.317</v>
+        <v>0.279</v>
       </c>
       <c r="P30" s="3" t="n">
         <v>0</v>
@@ -7994,7 +8102,7 @@
         <v>0</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>0.016</v>
+        <v>0.012</v>
       </c>
       <c r="P31" s="3" t="n">
         <v>0</v>
@@ -8058,7 +8166,7 @@
         <v>0</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>0.016</v>
+        <v>0.012</v>
       </c>
       <c r="P32" s="3" t="n">
         <v>0.048</v>
@@ -8122,7 +8230,7 @@
         <v>0</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>-0.016</v>
+        <v>-0.012</v>
       </c>
       <c r="P33" s="3" t="n">
         <v>-0.078</v>
@@ -8179,14 +8287,14 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>50–70 м</t>
+          <t>250–350 м</t>
         </is>
       </c>
       <c r="N34" s="3" t="n">
-        <v>-0.057</v>
+        <v>-0.109</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>0.139</v>
+        <v>0.124</v>
       </c>
       <c r="P34" s="3" t="n">
         <v>0</v>
@@ -8243,14 +8351,14 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>30–70 м</t>
+          <t>150–350 м</t>
         </is>
       </c>
       <c r="N35" s="3" t="n">
-        <v>0.05</v>
+        <v>-0.057</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>0.14</v>
+        <v>0.143</v>
       </c>
       <c r="P35" s="3" t="n">
         <v>0</v>
@@ -8307,7 +8415,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>50–70 м</t>
+          <t>250–350 м</t>
         </is>
       </c>
       <c r="N36" s="3" t="inlineStr"/>
@@ -8325,7 +8433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:T12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8347,6 +8455,7 @@
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8445,654 +8554,692 @@
           <t>MK18</t>
         </is>
       </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>Benelli M4</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>1.382</v>
+        <v>1.25</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1.396</v>
+        <v>1.266</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1.41</v>
+        <v>1.22</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>1.382</v>
+        <v>1.613</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>1.41</v>
+        <v>1.351</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>1.425</v>
+        <v>1.351</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>1.458</v>
+        <v>1.724</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>1.396</v>
+        <v>1.613</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>1.044</v>
+        <v>0.952</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>1.072</v>
+        <v>0.952</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>1.128</v>
+        <v>1</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>1.157</v>
+        <v>1</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>1.439</v>
+        <v>1.37</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>1.453</v>
+        <v>1.333</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>1.467</v>
+        <v>1.111</v>
       </c>
       <c r="Q2" s="3" t="n">
-        <v>1.594</v>
+        <v>1</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>1.636</v>
+        <v>0.87</v>
       </c>
       <c r="S2" s="3" t="n">
-        <v>1.458</v>
+        <v>1.724</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>1.389</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>1.298</v>
+        <v>1.147</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>1.289</v>
+        <v>1.176</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.302</v>
+        <v>1.157</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1.333</v>
+        <v>1.429</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>1.302</v>
+        <v>1.256</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>1.315</v>
+        <v>1.256</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>1.346</v>
+        <v>1.515</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>1.347</v>
+        <v>1.429</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.963</v>
+        <v>1.01</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>0.989</v>
+        <v>1.01</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1.041</v>
+        <v>1.064</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>1.067</v>
+        <v>1.064</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>1.328</v>
+        <v>1.279</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>1.341</v>
+        <v>1.272</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>1.354</v>
+        <v>1.19</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>1.471</v>
+        <v>1.078</v>
       </c>
       <c r="R3" s="3" t="n">
-        <v>1.51</v>
+        <v>0.917</v>
       </c>
       <c r="S3" s="3" t="n">
-        <v>1.346</v>
+        <v>1.515</v>
+      </c>
+      <c r="T3" s="3" t="n">
+        <v>0.317</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1.232</v>
+        <v>1.059</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1.25</v>
+        <v>1.099</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.242</v>
+        <v>1.101</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1.243</v>
+        <v>1.282</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1.263</v>
+        <v>1.174</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>1.276</v>
+        <v>1.174</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>1.255</v>
+        <v>1.351</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1.256</v>
+        <v>1.282</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.899</v>
+        <v>1.075</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.923</v>
+        <v>1.075</v>
       </c>
       <c r="L4" s="3" t="n">
+        <v>1.136</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>1.136</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>1.199</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>1.217</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>1.282</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>1.168</v>
+      </c>
+      <c r="R4" s="3" t="n">
         <v>0.971</v>
       </c>
-      <c r="M4" s="3" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="N4" s="3" t="n">
-        <v>1.266</v>
-      </c>
-      <c r="O4" s="3" t="n">
-        <v>1.251</v>
-      </c>
-      <c r="P4" s="3" t="n">
-        <v>1.263</v>
-      </c>
-      <c r="Q4" s="3" t="n">
-        <v>1.372</v>
-      </c>
-      <c r="R4" s="3" t="n">
-        <v>1.409</v>
-      </c>
       <c r="S4" s="3" t="n">
-        <v>1.255</v>
+        <v>1.351</v>
+      </c>
+      <c r="T4" s="3" t="n">
+        <v>0.167</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1.089</v>
+        <v>0.973</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1.105</v>
+        <v>1.025</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1.122</v>
+        <v>1.037</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1.099</v>
+        <v>1.035</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>1.116</v>
+        <v>1.101</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>1.128</v>
+        <v>1.101</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>1.095</v>
+        <v>1.027</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>1.111</v>
+        <v>1.035</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.8120000000000001</v>
+        <v>1.152</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>0.834</v>
+        <v>1.152</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>0.859</v>
+        <v>1.232</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>0.88</v>
+        <v>1.232</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>1.144</v>
+        <v>1.121</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>1.161</v>
+        <v>1.147</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>1.144</v>
+        <v>1.37</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>1.213</v>
+        <v>1.295</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>1.245</v>
+        <v>1.064</v>
       </c>
       <c r="S5" s="3" t="n">
-        <v>1.095</v>
+        <v>1.027</v>
+      </c>
+      <c r="T5" s="3" t="n">
+        <v>0.143</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0.948</v>
+        <v>0.89</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.962</v>
+        <v>0.954</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.976</v>
+        <v>0.969</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.947</v>
+        <v>0.795</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.972</v>
+        <v>1.037</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.982</v>
+        <v>1.037</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.928</v>
+        <v>0.734</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.956</v>
+        <v>0.795</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.723</v>
+        <v>1.244</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0.742</v>
+        <v>1.244</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>0.781</v>
+        <v>1.359</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.801</v>
+        <v>1.359</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>0.996</v>
+        <v>1.046</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>1.011</v>
+        <v>1.068</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>1.02</v>
+        <v>1.449</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>1.08</v>
+        <v>1.479</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>1.084</v>
+        <v>1.22</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>0.928</v>
+        <v>0.734</v>
+      </c>
+      <c r="T6" s="3" t="n">
+        <v>0.125</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0.847</v>
+        <v>0.82</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.868</v>
+        <v>0.893</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0.881</v>
+        <v>0.909</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.835</v>
+        <v>0.645</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.876</v>
+        <v>0.98</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0.885</v>
+        <v>0.98</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.826</v>
+        <v>0.571</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>0.844</v>
+        <v>0.645</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.652</v>
+        <v>1.351</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0.669</v>
+        <v>1.351</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>0.704</v>
+        <v>1.515</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.722</v>
+        <v>1.515</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>0.898</v>
+        <v>0.98</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.911</v>
+        <v>1</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>0.92</v>
+        <v>1.538</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>0.995</v>
+        <v>1.724</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>0.99</v>
+        <v>1.429</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>0.826</v>
+        <v>0.571</v>
+      </c>
+      <c r="T7" s="3" t="n">
+        <v>0.111</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>60</v>
+        <v>300</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0.671</v>
+        <v>0.746</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.71</v>
+        <v>0.847</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.666</v>
+        <v>0.488</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.7</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.707</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.666</v>
+        <v>0.426</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0.672</v>
+        <v>0.488</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.525</v>
+        <v>1.295</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0.539</v>
+        <v>1.295</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>0.5679999999999999</v>
+        <v>1.479</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.582</v>
+        <v>1.479</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.724</v>
+        <v>0.923</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.734</v>
+        <v>0.962</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>0.742</v>
+        <v>1.348</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>0.802</v>
+        <v>1.592</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>0.819</v>
+        <v>1.613</v>
       </c>
       <c r="S8" s="3" t="n">
-        <v>0.666</v>
+        <v>0.426</v>
+      </c>
+      <c r="T8" s="3" t="n">
+        <v>0.104</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>70</v>
+        <v>350</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.57</v>
+        <v>0.753</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.583</v>
+        <v>0.794</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.392</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.576</v>
+        <v>0.909</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0.581</v>
+        <v>0.909</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.339</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.392</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.441</v>
+        <v>1.244</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>0.453</v>
+        <v>1.244</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>0.476</v>
+        <v>1.445</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.488</v>
+        <v>1.445</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.594</v>
+        <v>0.871</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.609</v>
+        <v>0.926</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>0.622</v>
+        <v>1.199</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>0.673</v>
+        <v>1.479</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>0.6870000000000001</v>
+        <v>1.852</v>
       </c>
       <c r="S9" s="3" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.339</v>
+      </c>
+      <c r="T9" s="3" t="n">
+        <v>0.098</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>80</v>
+        <v>400</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0.468</v>
+        <v>0.623</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.473</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.478</v>
+        <v>0.73</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.468</v>
+        <v>0.323</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.478</v>
+        <v>0.85</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.483</v>
+        <v>0.85</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.468</v>
+        <v>0.278</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.473</v>
+        <v>0.323</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.366</v>
+        <v>1.092</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.375</v>
+        <v>1.092</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.399</v>
+        <v>1.299</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.409</v>
+        <v>1.299</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.487</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.498</v>
+        <v>0.862</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>0.516</v>
+        <v>1.006</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>0.5639999999999999</v>
+        <v>1.25</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>0.576</v>
+        <v>1.908</v>
       </c>
       <c r="S10" s="3" t="n">
-        <v>0.468</v>
+        <v>0.278</v>
+      </c>
+      <c r="T10" s="3" t="n">
+        <v>0.093</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>90</v>
+        <v>450</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>0.394</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.398</v>
+        <v>0.631</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.402</v>
+        <v>0.662</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.394</v>
+        <v>0.27</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.402</v>
+        <v>0.776</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.406</v>
+        <v>0.776</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.394</v>
+        <v>0.233</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.398</v>
+        <v>0.27</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.301</v>
+        <v>0.903</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.309</v>
+        <v>0.903</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>0.329</v>
+        <v>1.099</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.337</v>
+        <v>1.099</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.41</v>
+        <v>0.745</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.414</v>
+        <v>0.781</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>0.424</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>0.468</v>
+        <v>1</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>0.485</v>
+        <v>1.748</v>
       </c>
       <c r="S11" s="3" t="n">
-        <v>0.394</v>
+        <v>0.233</v>
+      </c>
+      <c r="T11" s="3" t="n">
+        <v>0.08799999999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.341</v>
+        <v>0.513</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.344</v>
+        <v>0.581</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.348</v>
+        <v>0.606</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.341</v>
+        <v>0.233</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.348</v>
+        <v>0.714</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.351</v>
+        <v>0.714</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.341</v>
+        <v>0.2</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.344</v>
+        <v>0.233</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.257</v>
+        <v>0.769</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.264</v>
+        <v>0.769</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0.278</v>
+        <v>0.952</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.285</v>
+        <v>0.952</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.355</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.358</v>
+        <v>0.714</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.362</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>0.393</v>
+        <v>0.833</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>0.419</v>
+        <v>1.613</v>
       </c>
       <c r="S12" s="3" t="n">
-        <v>0.341</v>
+        <v>0.2</v>
+      </c>
+      <c r="T12" s="3" t="n">
+        <v>0.083</v>
       </c>
     </row>
   </sheetData>
@@ -9107,7 +9254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:T12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -9129,6 +9276,7 @@
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9227,6 +9375,11 @@
           <t>MK18</t>
         </is>
       </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>Benelli M4</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -9286,10 +9439,13 @@
       <c r="S2" s="3" t="n">
         <v>0.239</v>
       </c>
+      <c r="T2" s="3" t="n">
+        <v>0.336</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>0.372</v>
@@ -9345,10 +9501,13 @@
       <c r="S3" s="3" t="n">
         <v>0.256</v>
       </c>
+      <c r="T3" s="3" t="n">
+        <v>0.76</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>0.428</v>
@@ -9404,10 +9563,13 @@
       <c r="S4" s="3" t="n">
         <v>0.272</v>
       </c>
+      <c r="T4" s="3" t="n">
+        <v>1.344</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>0.531</v>
@@ -9463,10 +9625,13 @@
       <c r="S5" s="3" t="n">
         <v>0.357</v>
       </c>
+      <c r="T5" s="3" t="n">
+        <v>1.557</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0.681</v>
@@ -9522,10 +9687,13 @@
       <c r="S6" s="3" t="n">
         <v>0.51</v>
       </c>
+      <c r="T6" s="3" t="n">
+        <v>1.771</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>0.832</v>
@@ -9581,10 +9749,13 @@
       <c r="S7" s="3" t="n">
         <v>0.663</v>
       </c>
+      <c r="T7" s="3" t="n">
+        <v>1.984</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>60</v>
+        <v>300</v>
       </c>
       <c r="B8" s="3" t="n">
         <v>1.001</v>
@@ -9640,10 +9811,13 @@
       <c r="S8" s="3" t="n">
         <v>0.829</v>
       </c>
+      <c r="T8" s="3" t="n">
+        <v>2.131</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>70</v>
+        <v>350</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>1.17</v>
@@ -9699,10 +9873,13 @@
       <c r="S9" s="3" t="n">
         <v>0.996</v>
       </c>
+      <c r="T9" s="3" t="n">
+        <v>2.278</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>80</v>
+        <v>400</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>1.337</v>
@@ -9758,10 +9935,13 @@
       <c r="S10" s="3" t="n">
         <v>1.167</v>
       </c>
+      <c r="T10" s="3" t="n">
+        <v>2.426</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>90</v>
+        <v>450</v>
       </c>
       <c r="B11" s="3" t="n">
         <v>1.503</v>
@@ -9817,10 +9997,13 @@
       <c r="S11" s="3" t="n">
         <v>1.344</v>
       </c>
+      <c r="T11" s="3" t="n">
+        <v>2.573</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>1.67</v>
@@ -9875,6 +10058,9 @@
       </c>
       <c r="S12" s="3" t="n">
         <v>1.521</v>
+      </c>
+      <c r="T12" s="3" t="n">
+        <v>2.72</v>
       </c>
     </row>
   </sheetData>
@@ -9889,7 +10075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:T11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -9911,6 +10097,7 @@
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10009,6 +10196,11 @@
           <t>MK18</t>
         </is>
       </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>Benelli M4</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -10067,6 +10259,9 @@
       </c>
       <c r="S2" s="3" t="n">
         <v>1.667</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>0.8</v>
       </c>
     </row>
     <row r="3">
@@ -10127,6 +10322,9 @@
       <c r="S3" s="3" t="n">
         <v>0.747</v>
       </c>
+      <c r="T3" s="3" t="n">
+        <v>0.299</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -10186,6 +10384,9 @@
       <c r="S4" s="3" t="n">
         <v>0.433</v>
       </c>
+      <c r="T4" s="3" t="n">
+        <v>0.16</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -10245,6 +10446,9 @@
       <c r="S5" s="3" t="n">
         <v>0.244</v>
       </c>
+      <c r="T5" s="3" t="n">
+        <v>0.08799999999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -10304,6 +10508,9 @@
       <c r="S6" s="3" t="n">
         <v>0.157</v>
       </c>
+      <c r="T6" s="3" t="n">
+        <v>0.056</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -10363,6 +10570,9 @@
       <c r="S7" s="3" t="n">
         <v>0.109</v>
       </c>
+      <c r="T7" s="3" t="n">
+        <v>0.039</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -10422,6 +10632,9 @@
       <c r="S8" s="3" t="n">
         <v>0.076</v>
       </c>
+      <c r="T8" s="3" t="n">
+        <v>0.027</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -10481,6 +10694,9 @@
       <c r="S9" s="3" t="n">
         <v>0.056</v>
       </c>
+      <c r="T9" s="3" t="n">
+        <v>0.02</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -10540,6 +10756,9 @@
       <c r="S10" s="3" t="n">
         <v>0.043</v>
       </c>
+      <c r="T10" s="3" t="n">
+        <v>0.015</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -10598,6 +10817,9 @@
       </c>
       <c r="S11" s="3" t="n">
         <v>0.034</v>
+      </c>
+      <c r="T11" s="3" t="n">
+        <v>0.012</v>
       </c>
     </row>
   </sheetData>
@@ -10745,648 +10967,648 @@
         <v>0</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>1.439</v>
+        <v>1.37</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>1.285</v>
+        <v>1.223</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.468</v>
+        <v>1.398</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1.468</v>
+        <v>1.398</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>1.384</v>
+        <v>1.317</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>1.564</v>
+        <v>1.489</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>1.599</v>
+        <v>1.522</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>1.599</v>
+        <v>1.522</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>1.564</v>
+        <v>1.489</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>1.581</v>
+        <v>1.505</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1.564</v>
+        <v>1.489</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>1.564</v>
+        <v>1.489</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>1.285</v>
+        <v>1.223</v>
       </c>
       <c r="O3" s="3" t="n">
-        <v>1.124</v>
+        <v>1.07</v>
       </c>
       <c r="P3" s="3" t="n">
-        <v>1.074</v>
+        <v>1.022</v>
       </c>
       <c r="Q3" s="3" t="n">
-        <v>1.028</v>
+        <v>0.978</v>
       </c>
       <c r="R3" s="3" t="n">
-        <v>1.308</v>
+        <v>1.245</v>
       </c>
       <c r="S3" s="3" t="n">
-        <v>1.357</v>
+        <v>1.292</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1.328</v>
+        <v>1.279</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1.222</v>
+        <v>1.177</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.383</v>
+        <v>1.332</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1.398</v>
+        <v>1.346</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1.355</v>
+        <v>1.305</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>1.433</v>
+        <v>1.38</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>1.498</v>
+        <v>1.279</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1.454</v>
+        <v>1.279</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>1.465</v>
+        <v>1.41</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>1.449</v>
+        <v>1.395</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>1.436</v>
+        <v>1.382</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>1.454</v>
+        <v>1.4</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>1.229</v>
+        <v>1.184</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>1.08</v>
+        <v>1.04</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>1.034</v>
+        <v>0.996</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>0.988</v>
+        <v>0.952</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>1.229</v>
+        <v>1.184</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>1.289</v>
+        <v>1.242</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1.266</v>
+        <v>1.199</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1.202</v>
+        <v>1.138</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1.347</v>
+        <v>1.276</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1.377</v>
+        <v>1.303</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>1.347</v>
+        <v>1.276</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>1.347</v>
+        <v>1.276</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>1.407</v>
+        <v>1.199</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>1.319</v>
+        <v>1.199</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>1.347</v>
+        <v>1.276</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>1.333</v>
+        <v>1.262</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>1.362</v>
+        <v>1.289</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>1.34</v>
+        <v>1.269</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>1.319</v>
+        <v>1.249</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>1.073</v>
+        <v>1.016</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>1.031</v>
+        <v>0.976</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>0.984</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>1.195</v>
+        <v>1.131</v>
       </c>
       <c r="S5" s="3" t="n">
-        <v>1.288</v>
+        <v>1.219</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1.144</v>
+        <v>1.121</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1.122</v>
+        <v>1.099</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.257</v>
+        <v>1.232</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>1.262</v>
+        <v>1.236</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>1.264</v>
+        <v>1.239</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>1.137</v>
+        <v>1.114</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>1.192</v>
+        <v>1.121</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>1.144</v>
+        <v>1.121</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>1.137</v>
+        <v>1.114</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>1.137</v>
+        <v>1.114</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>1.172</v>
+        <v>1.148</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>1.137</v>
+        <v>1.114</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>1.286</v>
+        <v>1.26</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>1.013</v>
+        <v>0.992</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>0.976</v>
+        <v>0.957</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>0.93</v>
+        <v>0.911</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>1.1</v>
+        <v>1.078</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>1.2</v>
+        <v>1.176</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0.996</v>
+        <v>1.046</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>1.132</v>
+        <v>1.189</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1.132</v>
+        <v>1.189</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>1.048</v>
+        <v>1.101</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>1.138</v>
+        <v>1.195</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>1.016</v>
+        <v>1.067</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.996</v>
+        <v>1.046</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>0.996</v>
+        <v>1.046</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.987</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.987</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>0.976</v>
+        <v>1.026</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.987</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>1.215</v>
+        <v>1.276</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.922</v>
+        <v>0.969</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>0.892</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="Q7" s="3" t="n">
-        <v>0.849</v>
+        <v>0.891</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>1.107</v>
+        <v>1.162</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>1.06</v>
+        <v>1.113</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0.898</v>
+        <v>0.98</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>1.069</v>
+        <v>1.167</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>1.069</v>
+        <v>1.167</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.881</v>
+        <v>0.961</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>1.036</v>
+        <v>1.131</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.987</v>
+        <v>1.077</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.898</v>
+        <v>0.98</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0.898</v>
+        <v>0.98</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.824</v>
+        <v>0.899</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0.824</v>
+        <v>0.899</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>0.847</v>
+        <v>0.925</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.824</v>
+        <v>0.899</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>1.044</v>
+        <v>1.14</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.916</v>
+        <v>1</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>0.847</v>
+        <v>0.925</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>0.804</v>
+        <v>0.878</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>1.044</v>
+        <v>1.14</v>
       </c>
       <c r="S8" s="3" t="n">
-        <v>0.966</v>
+        <v>1.054</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>60</v>
+        <v>300</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0.724</v>
+        <v>0.923</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.823</v>
+        <v>1.048</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.835</v>
+        <v>1.064</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.87</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.823</v>
+        <v>1.048</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0.791</v>
+        <v>1.008</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.724</v>
+        <v>0.923</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>0.724</v>
+        <v>0.923</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.646</v>
+        <v>0.824</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>0.646</v>
+        <v>0.824</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>0.67</v>
+        <v>0.854</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.646</v>
+        <v>0.824</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>0.787</v>
+        <v>1.003</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>0.823</v>
+        <v>1.048</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>0.754</v>
+        <v>0.961</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.87</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>0.829</v>
+        <v>1.056</v>
       </c>
       <c r="S9" s="3" t="n">
-        <v>0.787</v>
+        <v>1.003</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>70</v>
+        <v>350</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0.594</v>
+        <v>0.871</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.649</v>
+        <v>0.952</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.66</v>
+        <v>0.968</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.646</v>
+        <v>0.947</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.629</v>
+        <v>0.922</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.594</v>
+        <v>0.871</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.594</v>
+        <v>0.871</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.528</v>
+        <v>0.774</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.528</v>
+        <v>0.774</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.54</v>
+        <v>0.792</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.528</v>
+        <v>0.774</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.594</v>
+        <v>0.871</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.6909999999999999</v>
+        <v>1.013</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>0.6909999999999999</v>
+        <v>1.013</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>0.613</v>
+        <v>0.898</v>
       </c>
       <c r="R10" s="3" t="n">
-        <v>0.664</v>
+        <v>0.973</v>
       </c>
       <c r="S10" s="3" t="n">
-        <v>0.626</v>
+        <v>0.917</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>80</v>
+        <v>400</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>0.487</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.516</v>
+        <v>0.858</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.518</v>
+        <v>0.862</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.455</v>
+        <v>0.757</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.508</v>
+        <v>0.844</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.499</v>
+        <v>0.83</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.487</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.487</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.431</v>
+        <v>0.717</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.431</v>
+        <v>0.717</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>0.44</v>
+        <v>0.732</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.431</v>
+        <v>0.717</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.462</v>
+        <v>0.767</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.542</v>
+        <v>0.9</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>0.58</v>
+        <v>0.965</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>0.554</v>
+        <v>0.921</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>0.527</v>
+        <v>0.876</v>
       </c>
       <c r="S11" s="3" t="n">
-        <v>0.497</v>
+        <v>0.827</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>90</v>
+        <v>450</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.41</v>
+        <v>0.745</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.419</v>
+        <v>0.76</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.419</v>
+        <v>0.76</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.382</v>
+        <v>0.6929999999999999</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.406</v>
+        <v>0.738</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.407</v>
+        <v>0.739</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.41</v>
+        <v>0.745</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.41</v>
+        <v>0.745</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.362</v>
+        <v>0.657</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.362</v>
+        <v>0.657</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0.369</v>
+        <v>0.669</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.362</v>
+        <v>0.657</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.377</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.443</v>
+        <v>0.804</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.466</v>
+        <v>0.847</v>
       </c>
       <c r="Q12" s="3" t="n">
-        <v>0.472</v>
+        <v>0.857</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>0.428</v>
+        <v>0.776</v>
       </c>
       <c r="S12" s="3" t="n">
-        <v>0.402</v>
+        <v>0.731</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0.355</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.348</v>
+        <v>0.676</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.348</v>
+        <v>0.676</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.328</v>
+        <v>0.639</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.335</v>
+        <v>0.651</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>0.341</v>
+        <v>0.663</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.355</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>0.355</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.311</v>
+        <v>0.605</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>0.311</v>
+        <v>0.605</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>0.317</v>
+        <v>0.616</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.311</v>
+        <v>0.605</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.317</v>
+        <v>0.616</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.377</v>
+        <v>0.734</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>0.433</v>
+        <v>0.841</v>
       </c>
       <c r="Q13" s="3" t="n">
-        <v>0.412</v>
+        <v>0.802</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>0.355</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="S13" s="3" t="n">
-        <v>0.335</v>
+        <v>0.651</v>
       </c>
     </row>
   </sheetData>
@@ -11683,7 +11905,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>0.263</v>
@@ -11772,7 +11994,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>0.291</v>
@@ -11861,7 +12083,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0.355</v>
@@ -11950,7 +12172,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>0.454</v>
@@ -12039,7 +12261,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="B8" s="3" t="n">
         <v>0.553</v>
@@ -12128,7 +12350,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>60</v>
+        <v>300</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>0.674</v>
@@ -12217,7 +12439,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>70</v>
+        <v>350</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>0.795</v>
@@ -12306,7 +12528,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>80</v>
+        <v>400</v>
       </c>
       <c r="B11" s="3" t="n">
         <v>0.919</v>
@@ -12395,7 +12617,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>90</v>
+        <v>450</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>1.045</v>
@@ -12484,7 +12706,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="B13" s="3" t="n">
         <v>1.172</v>
@@ -13038,153 +13260,153 @@
         <v>0</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>1.41</v>
+        <v>1.351</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>1.41</v>
+        <v>1.351</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.331</v>
+        <v>1.275</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1.302</v>
+        <v>1.256</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1.302</v>
+        <v>1.256</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.255</v>
+        <v>1.211</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1.263</v>
+        <v>1.174</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1.263</v>
+        <v>1.174</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1.245</v>
+        <v>1.157</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1.116</v>
+        <v>1.101</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1.109</v>
+        <v>1.094</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.126</v>
+        <v>1.111</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>40</v>
+        <v>200</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0.972</v>
+        <v>1.037</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.953</v>
+        <v>1.017</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1.034</v>
+        <v>1.104</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0.876</v>
+        <v>0.98</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.843</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>1.019</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>60</v>
+        <v>300</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0.7</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.66</v>
+        <v>0.89</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.833</v>
+        <v>1.123</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>70</v>
+        <v>350</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0.576</v>
+        <v>0.909</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.538</v>
+        <v>0.85</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.654</v>
+        <v>1.033</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>80</v>
+        <v>400</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>0.478</v>
+        <v>0.85</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.442</v>
+        <v>0.787</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.526</v>
+        <v>0.9360000000000001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>90</v>
+        <v>450</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.402</v>
+        <v>0.776</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.369</v>
+        <v>0.712</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.435</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0.348</v>
+        <v>0.714</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.316</v>
+        <v>0.649</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.37</v>
+        <v>0.76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalize weapon combat and animation updates
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Tools/CombatBalanceParameters.xlsx
+++ b/Tools/CombatBalanceParameters.xlsx
@@ -18,6 +18,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AK точность" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AK прицел" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AK отдача" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SVD прицел" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SVD отдача" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sniper прицел" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sniper отдача" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -788,6 +792,166 @@
             </numRef>
           </val>
         </ser>
+        <ser>
+          <idx val="19"/>
+          <order val="19"/>
+          <tx>
+            <strRef>
+              <f>'Точность'!U1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Точность'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Точность'!$U$2:$U$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="20"/>
+          <order val="20"/>
+          <tx>
+            <strRef>
+              <f>'Точность'!V1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Точность'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Точность'!$V$2:$V$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="21"/>
+          <order val="21"/>
+          <tx>
+            <strRef>
+              <f>'Точность'!W1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Точность'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Точность'!$W$2:$W$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="22"/>
+          <order val="22"/>
+          <tx>
+            <strRef>
+              <f>'Точность'!X1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Точность'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Точность'!$X$2:$X$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="23"/>
+          <order val="23"/>
+          <tx>
+            <strRef>
+              <f>'Точность'!Y1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Точность'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Точность'!$Y$2:$Y$12</f>
+            </numRef>
+          </val>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -834,6 +998,606 @@
                 </a:pPr>
                 <a:r>
                   <a:t>Качество точности</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SVD прицел</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'SVD прицел'!B2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'SVD прицел'!$A$3:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'SVD прицел'!$B$3:$B$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'SVD прицел'!C2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'SVD прицел'!$A$3:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'SVD прицел'!$C$3:$C$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Дист, м</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Время, сек</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SVD отдача</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'SVD отдача'!B2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'SVD отдача'!$A$3:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'SVD отдача'!$B$3:$B$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'SVD отдача'!C2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'SVD отдача'!$A$3:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'SVD отдача'!$C$3:$C$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Выстрел</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Контроль отдачи</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Sniper прицел</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Sniper прицел'!B2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sniper прицел'!$A$3:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sniper прицел'!$B$3:$B$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Sniper прицел'!C2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sniper прицел'!$A$3:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sniper прицел'!$C$3:$C$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Дист, м</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Время, сек</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Sniper отдача</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Sniper отдача'!B2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sniper отдача'!$A$3:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sniper отдача'!$B$3:$B$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Sniper отдача'!C2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Sniper отдача'!$A$3:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Sniper отдача'!$C$3:$C$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Выстрел</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Контроль отдачи</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1482,6 +2246,166 @@
             </numRef>
           </val>
         </ser>
+        <ser>
+          <idx val="19"/>
+          <order val="19"/>
+          <tx>
+            <strRef>
+              <f>'Прицеливание'!U1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Прицеливание'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Прицеливание'!$U$2:$U$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="20"/>
+          <order val="20"/>
+          <tx>
+            <strRef>
+              <f>'Прицеливание'!V1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Прицеливание'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Прицеливание'!$V$2:$V$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="21"/>
+          <order val="21"/>
+          <tx>
+            <strRef>
+              <f>'Прицеливание'!W1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Прицеливание'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Прицеливание'!$W$2:$W$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="22"/>
+          <order val="22"/>
+          <tx>
+            <strRef>
+              <f>'Прицеливание'!X1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Прицеливание'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Прицеливание'!$X$2:$X$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="23"/>
+          <order val="23"/>
+          <tx>
+            <strRef>
+              <f>'Прицеливание'!Y1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Прицеливание'!$A$2:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Прицеливание'!$Y$2:$Y$12</f>
+            </numRef>
+          </val>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -2176,6 +3100,166 @@
             </numRef>
           </val>
         </ser>
+        <ser>
+          <idx val="19"/>
+          <order val="19"/>
+          <tx>
+            <strRef>
+              <f>'Отдача'!U1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Отдача'!$A$2:$A$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Отдача'!$U$2:$U$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="20"/>
+          <order val="20"/>
+          <tx>
+            <strRef>
+              <f>'Отдача'!V1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Отдача'!$A$2:$A$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Отдача'!$V$2:$V$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="21"/>
+          <order val="21"/>
+          <tx>
+            <strRef>
+              <f>'Отдача'!W1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Отдача'!$A$2:$A$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Отдача'!$W$2:$W$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="22"/>
+          <order val="22"/>
+          <tx>
+            <strRef>
+              <f>'Отдача'!X1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Отдача'!$A$2:$A$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Отдача'!$X$2:$X$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="23"/>
+          <order val="23"/>
+          <tx>
+            <strRef>
+              <f>'Отдача'!Y1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Отдача'!$A$2:$A$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Отдача'!$Y$2:$Y$11</f>
+            </numRef>
+          </val>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -4376,6 +5460,38 @@
             </numRef>
           </val>
         </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'AK точность'!E2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'AK точность'!$A$3:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'AK точность'!$E$3:$E$13</f>
+            </numRef>
+          </val>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -4622,6 +5738,38 @@
             </numRef>
           </val>
         </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'AK прицел'!G2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'AK прицел'!$A$3:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'AK прицел'!$G$3:$G$13</f>
+            </numRef>
+          </val>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -4876,6 +6024,114 @@
       <col>0</col>
       <colOff>0</colOff>
       <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="4320000"/>
@@ -5607,7 +6863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5616,6 +6872,7 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5656,6 +6913,11 @@
           <t>+ SilencerAK 545</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>+ Scope8</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -5676,6 +6938,9 @@
       <c r="F3" s="3" t="n">
         <v>0.284</v>
       </c>
+      <c r="G3" s="3" t="n">
+        <v>0.422</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -5696,6 +6961,9 @@
       <c r="F4" s="3" t="n">
         <v>0.328</v>
       </c>
+      <c r="G4" s="3" t="n">
+        <v>0.472</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -5716,6 +6984,9 @@
       <c r="F5" s="3" t="n">
         <v>0.372</v>
       </c>
+      <c r="G5" s="3" t="n">
+        <v>0.518</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -5736,6 +7007,9 @@
       <c r="F6" s="3" t="n">
         <v>0.451</v>
       </c>
+      <c r="G6" s="3" t="n">
+        <v>0.608</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -5756,6 +7030,9 @@
       <c r="F7" s="3" t="n">
         <v>0.5659999999999999</v>
       </c>
+      <c r="G7" s="3" t="n">
+        <v>0.697</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -5776,6 +7053,9 @@
       <c r="F8" s="3" t="n">
         <v>0.68</v>
       </c>
+      <c r="G8" s="3" t="n">
+        <v>0.775</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -5796,6 +7076,9 @@
       <c r="F9" s="3" t="n">
         <v>0.8139999999999999</v>
       </c>
+      <c r="G9" s="3" t="n">
+        <v>0.914</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -5816,6 +7099,9 @@
       <c r="F10" s="3" t="n">
         <v>0.948</v>
       </c>
+      <c r="G10" s="3" t="n">
+        <v>1.062</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -5836,6 +7122,9 @@
       <c r="F11" s="3" t="n">
         <v>1.082</v>
       </c>
+      <c r="G11" s="3" t="n">
+        <v>1.225</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -5856,6 +7145,9 @@
       <c r="F12" s="3" t="n">
         <v>1.217</v>
       </c>
+      <c r="G12" s="3" t="n">
+        <v>1.404</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -5876,10 +7168,13 @@
       <c r="F13" s="3" t="n">
         <v>1.351</v>
       </c>
+      <c r="G13" s="3" t="n">
+        <v>1.602</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6079,13 +7374,663 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Эталон: SVD. Каждый столбец = базовое оружие + один модуль.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Дист, м</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>База (SVD)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>+ SVD Silencer</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.756</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.716</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>100</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.675</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>150</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.657</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.6889999999999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>200</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.722</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.758</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>250</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0.787</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.827</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>300</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0.839</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0.881</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>350</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0.891</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>400</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>1.019</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>450</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1.078</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>1.132</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>500</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>1.186</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1.245</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Эталон: SVD. Каждый столбец = базовое оружие + один модуль.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Выстрел</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>База (SVD)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>+ SVD MuzzleBrake</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>2.174</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1.89</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>1.976</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1.719</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1.787</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1.554</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1.418</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>1.304</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>1.328</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1.154</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1.191</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>1.036</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>0.9389999999999999</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0.988</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>0.859</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Эталон: Sniper 7.62x51. Каждый столбец = базовое оружие + один модуль.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Дист, м</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>База (Sniper 7.62x51)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>+ Sniper762 Silencer</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.946</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.993</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>100</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.947</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>150</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.895</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>200</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.926</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.973</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>250</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>1.005</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>300</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0.9370000000000001</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0.984</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>350</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.963</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>400</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0.928</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>0.975</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>450</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>1.019</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>500</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>1.012</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1.063</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Эталон: Sniper 7.62x51. Каждый столбец = базовое оружие + один модуль.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Выстрел</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>База (Sniper 7.62x51)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>+ Sniper762 MuzzleBrake</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>2.381</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2.126</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2.289</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2.044</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>2.205</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1.968</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>2.053</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1.833</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1.714</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>1.804</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>1.61</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>1.625</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1.451</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1.479</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>1.32</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1.357</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>1.211</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1.253</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>1.119</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:P40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8372,7 +10317,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>AK</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -8418,9 +10363,271 @@
           <t>250–350 м</t>
         </is>
       </c>
-      <c r="N36" s="3" t="inlineStr"/>
-      <c r="O36" s="3" t="inlineStr"/>
-      <c r="P36" s="3" t="inlineStr"/>
+      <c r="N36" s="3" t="n">
+        <v>-0.163</v>
+      </c>
+      <c r="O36" s="3" t="n">
+        <v>0.156</v>
+      </c>
+      <c r="P36" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sniper762 MuzzleBrake</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Sniper</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Compensator</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Muzzle</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="I37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>нейтральный</t>
+        </is>
+      </c>
+      <c r="N37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" s="3" t="n">
+        <v>-0.206</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Sniper762 Silencer</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Sniper</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Suppressor</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Muzzle</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>нейтральный</t>
+        </is>
+      </c>
+      <c r="N38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="3" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="P38" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SVD MuzzleBrake</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>SVD</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Compensator</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Muzzle</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="I39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>нейтральный</t>
+        </is>
+      </c>
+      <c r="N39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" s="3" t="n">
+        <v>-0.213</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SVD Silencer</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>SVD</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Suppressor</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Muzzle</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>нейтральный</t>
+        </is>
+      </c>
+      <c r="N40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="3" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="P40" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8433,7 +10640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T12"/>
+  <dimension ref="A1:Y12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8456,6 +10663,11 @@
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8559,6 +10771,31 @@
           <t>Benelli M4</t>
         </is>
       </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>Mosin</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>SVD</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>Sniper 7.62x51</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>M249</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>PKM</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -8621,6 +10858,21 @@
       <c r="T2" s="3" t="n">
         <v>1.389</v>
       </c>
+      <c r="U2" s="3" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>0.952</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -8683,6 +10935,21 @@
       <c r="T3" s="3" t="n">
         <v>0.317</v>
       </c>
+      <c r="U3" s="3" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>1.078</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="X3" s="3" t="n">
+        <v>1.064</v>
+      </c>
+      <c r="Y3" s="3" t="n">
+        <v>1.01</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -8745,6 +11012,21 @@
       <c r="T4" s="3" t="n">
         <v>0.167</v>
       </c>
+      <c r="U4" s="3" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="V4" s="3" t="n">
+        <v>1.168</v>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>1.136</v>
+      </c>
+      <c r="Y4" s="3" t="n">
+        <v>1.075</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -8807,6 +11089,21 @@
       <c r="T5" s="3" t="n">
         <v>0.143</v>
       </c>
+      <c r="U5" s="3" t="n">
+        <v>1.064</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>1.295</v>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>1.064</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>1.232</v>
+      </c>
+      <c r="Y5" s="3" t="n">
+        <v>1.152</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -8869,6 +11166,21 @@
       <c r="T6" s="3" t="n">
         <v>0.125</v>
       </c>
+      <c r="U6" s="3" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="V6" s="3" t="n">
+        <v>1.479</v>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="X6" s="3" t="n">
+        <v>1.359</v>
+      </c>
+      <c r="Y6" s="3" t="n">
+        <v>1.244</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -8931,6 +11243,21 @@
       <c r="T7" s="3" t="n">
         <v>0.111</v>
       </c>
+      <c r="U7" s="3" t="n">
+        <v>1.429</v>
+      </c>
+      <c r="V7" s="3" t="n">
+        <v>1.724</v>
+      </c>
+      <c r="W7" s="3" t="n">
+        <v>1.429</v>
+      </c>
+      <c r="X7" s="3" t="n">
+        <v>1.515</v>
+      </c>
+      <c r="Y7" s="3" t="n">
+        <v>1.351</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -8993,6 +11320,21 @@
       <c r="T8" s="3" t="n">
         <v>0.104</v>
       </c>
+      <c r="U8" s="3" t="n">
+        <v>1.613</v>
+      </c>
+      <c r="V8" s="3" t="n">
+        <v>1.592</v>
+      </c>
+      <c r="W8" s="3" t="n">
+        <v>1.613</v>
+      </c>
+      <c r="X8" s="3" t="n">
+        <v>1.479</v>
+      </c>
+      <c r="Y8" s="3" t="n">
+        <v>1.295</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -9055,6 +11397,21 @@
       <c r="T9" s="3" t="n">
         <v>0.098</v>
       </c>
+      <c r="U9" s="3" t="n">
+        <v>1.852</v>
+      </c>
+      <c r="V9" s="3" t="n">
+        <v>1.479</v>
+      </c>
+      <c r="W9" s="3" t="n">
+        <v>1.852</v>
+      </c>
+      <c r="X9" s="3" t="n">
+        <v>1.445</v>
+      </c>
+      <c r="Y9" s="3" t="n">
+        <v>1.244</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -9117,6 +11474,21 @@
       <c r="T10" s="3" t="n">
         <v>0.093</v>
       </c>
+      <c r="U10" s="3" t="n">
+        <v>1.908</v>
+      </c>
+      <c r="V10" s="3" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="W10" s="3" t="n">
+        <v>1.908</v>
+      </c>
+      <c r="X10" s="3" t="n">
+        <v>1.299</v>
+      </c>
+      <c r="Y10" s="3" t="n">
+        <v>1.092</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -9179,6 +11551,21 @@
       <c r="T11" s="3" t="n">
         <v>0.08799999999999999</v>
       </c>
+      <c r="U11" s="3" t="n">
+        <v>1.748</v>
+      </c>
+      <c r="V11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="W11" s="3" t="n">
+        <v>1.748</v>
+      </c>
+      <c r="X11" s="3" t="n">
+        <v>1.099</v>
+      </c>
+      <c r="Y11" s="3" t="n">
+        <v>0.903</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -9240,6 +11627,21 @@
       </c>
       <c r="T12" s="3" t="n">
         <v>0.083</v>
+      </c>
+      <c r="U12" s="3" t="n">
+        <v>1.613</v>
+      </c>
+      <c r="V12" s="3" t="n">
+        <v>0.833</v>
+      </c>
+      <c r="W12" s="3" t="n">
+        <v>1.613</v>
+      </c>
+      <c r="X12" s="3" t="n">
+        <v>0.952</v>
+      </c>
+      <c r="Y12" s="3" t="n">
+        <v>0.769</v>
       </c>
     </row>
   </sheetData>
@@ -9254,7 +11656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T12"/>
+  <dimension ref="A1:Y12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -9277,6 +11679,11 @@
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9380,6 +11787,31 @@
           <t>Benelli M4</t>
         </is>
       </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>Mosin</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>SVD</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>Sniper 7.62x51</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>M249</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>PKM</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -9442,6 +11874,21 @@
       <c r="T2" s="3" t="n">
         <v>0.336</v>
       </c>
+      <c r="U2" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>0.775</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -9504,6 +11951,21 @@
       <c r="T3" s="3" t="n">
         <v>0.76</v>
       </c>
+      <c r="U3" s="3" t="n">
+        <v>0.946</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>0.946</v>
+      </c>
+      <c r="X3" s="3" t="n">
+        <v>0.678</v>
+      </c>
+      <c r="Y3" s="3" t="n">
+        <v>0.735</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -9566,6 +12028,21 @@
       <c r="T4" s="3" t="n">
         <v>1.344</v>
       </c>
+      <c r="U4" s="3" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="V4" s="3" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>0.636</v>
+      </c>
+      <c r="Y4" s="3" t="n">
+        <v>0.695</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -9628,6 +12105,21 @@
       <c r="T5" s="3" t="n">
         <v>1.557</v>
       </c>
+      <c r="U5" s="3" t="n">
+        <v>0.895</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>0.657</v>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>0.895</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>0.646</v>
+      </c>
+      <c r="Y5" s="3" t="n">
+        <v>0.709</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -9690,6 +12182,21 @@
       <c r="T6" s="3" t="n">
         <v>1.771</v>
       </c>
+      <c r="U6" s="3" t="n">
+        <v>0.926</v>
+      </c>
+      <c r="V6" s="3" t="n">
+        <v>0.722</v>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>0.926</v>
+      </c>
+      <c r="X6" s="3" t="n">
+        <v>0.709</v>
+      </c>
+      <c r="Y6" s="3" t="n">
+        <v>0.777</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -9752,6 +12259,21 @@
       <c r="T7" s="3" t="n">
         <v>1.984</v>
       </c>
+      <c r="U7" s="3" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="V7" s="3" t="n">
+        <v>0.787</v>
+      </c>
+      <c r="W7" s="3" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="X7" s="3" t="n">
+        <v>0.773</v>
+      </c>
+      <c r="Y7" s="3" t="n">
+        <v>0.845</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -9814,6 +12336,21 @@
       <c r="T8" s="3" t="n">
         <v>2.131</v>
       </c>
+      <c r="U8" s="3" t="n">
+        <v>0.9370000000000001</v>
+      </c>
+      <c r="V8" s="3" t="n">
+        <v>0.839</v>
+      </c>
+      <c r="W8" s="3" t="n">
+        <v>0.9370000000000001</v>
+      </c>
+      <c r="X8" s="3" t="n">
+        <v>0.821</v>
+      </c>
+      <c r="Y8" s="3" t="n">
+        <v>0.907</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -9876,6 +12413,21 @@
       <c r="T9" s="3" t="n">
         <v>2.278</v>
       </c>
+      <c r="U9" s="3" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="V9" s="3" t="n">
+        <v>0.891</v>
+      </c>
+      <c r="W9" s="3" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="X9" s="3" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="Y9" s="3" t="n">
+        <v>0.969</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -9938,6 +12490,21 @@
       <c r="T10" s="3" t="n">
         <v>2.426</v>
       </c>
+      <c r="U10" s="3" t="n">
+        <v>0.928</v>
+      </c>
+      <c r="V10" s="3" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="W10" s="3" t="n">
+        <v>0.928</v>
+      </c>
+      <c r="X10" s="3" t="n">
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="Y10" s="3" t="n">
+        <v>1.059</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -10000,6 +12567,21 @@
       <c r="T11" s="3" t="n">
         <v>2.573</v>
       </c>
+      <c r="U11" s="3" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="V11" s="3" t="n">
+        <v>1.078</v>
+      </c>
+      <c r="W11" s="3" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="X11" s="3" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="Y11" s="3" t="n">
+        <v>1.177</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -10061,6 +12643,21 @@
       </c>
       <c r="T12" s="3" t="n">
         <v>2.72</v>
+      </c>
+      <c r="U12" s="3" t="n">
+        <v>1.012</v>
+      </c>
+      <c r="V12" s="3" t="n">
+        <v>1.186</v>
+      </c>
+      <c r="W12" s="3" t="n">
+        <v>1.012</v>
+      </c>
+      <c r="X12" s="3" t="n">
+        <v>1.138</v>
+      </c>
+      <c r="Y12" s="3" t="n">
+        <v>1.295</v>
       </c>
     </row>
   </sheetData>
@@ -10075,7 +12672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:Y11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10098,6 +12695,11 @@
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10201,6 +12803,31 @@
           <t>Benelli M4</t>
         </is>
       </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>Mosin</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>SVD</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>Sniper 7.62x51</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>M249</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>PKM</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -10262,6 +12889,21 @@
       </c>
       <c r="T2" s="3" t="n">
         <v>0.8</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>2.273</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>2.174</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>2.381</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>1.923</v>
       </c>
     </row>
     <row r="3">
@@ -10325,6 +12967,21 @@
       <c r="T3" s="3" t="n">
         <v>0.299</v>
       </c>
+      <c r="U3" s="3" t="n">
+        <v>2.185</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>2.289</v>
+      </c>
+      <c r="X3" s="3" t="n">
+        <v>1.359</v>
+      </c>
+      <c r="Y3" s="3" t="n">
+        <v>1.253</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -10387,6 +13044,21 @@
       <c r="T4" s="3" t="n">
         <v>0.16</v>
       </c>
+      <c r="U4" s="3" t="n">
+        <v>2.104</v>
+      </c>
+      <c r="V4" s="3" t="n">
+        <v>1.976</v>
+      </c>
+      <c r="W4" s="3" t="n">
+        <v>2.205</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>1.005</v>
+      </c>
+      <c r="Y4" s="3" t="n">
+        <v>0.897</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -10449,6 +13121,21 @@
       <c r="T5" s="3" t="n">
         <v>0.08799999999999999</v>
       </c>
+      <c r="U5" s="3" t="n">
+        <v>1.959</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>1.787</v>
+      </c>
+      <c r="W5" s="3" t="n">
+        <v>2.053</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="Y5" s="3" t="n">
+        <v>0.664</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -10511,6 +13198,21 @@
       <c r="T6" s="3" t="n">
         <v>0.056</v>
       </c>
+      <c r="U6" s="3" t="n">
+        <v>1.833</v>
+      </c>
+      <c r="V6" s="3" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="W6" s="3" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="X6" s="3" t="n">
+        <v>0.594</v>
+      </c>
+      <c r="Y6" s="3" t="n">
+        <v>0.512</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -10573,6 +13275,21 @@
       <c r="T7" s="3" t="n">
         <v>0.039</v>
       </c>
+      <c r="U7" s="3" t="n">
+        <v>1.722</v>
+      </c>
+      <c r="V7" s="3" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="W7" s="3" t="n">
+        <v>1.804</v>
+      </c>
+      <c r="X7" s="3" t="n">
+        <v>0.479</v>
+      </c>
+      <c r="Y7" s="3" t="n">
+        <v>0.408</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -10635,6 +13352,21 @@
       <c r="T8" s="3" t="n">
         <v>0.027</v>
       </c>
+      <c r="U8" s="3" t="n">
+        <v>1.551</v>
+      </c>
+      <c r="V8" s="3" t="n">
+        <v>1.328</v>
+      </c>
+      <c r="W8" s="3" t="n">
+        <v>1.625</v>
+      </c>
+      <c r="X8" s="3" t="n">
+        <v>0.372</v>
+      </c>
+      <c r="Y8" s="3" t="n">
+        <v>0.312</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -10697,6 +13429,21 @@
       <c r="T9" s="3" t="n">
         <v>0.02</v>
       </c>
+      <c r="U9" s="3" t="n">
+        <v>1.412</v>
+      </c>
+      <c r="V9" s="3" t="n">
+        <v>1.191</v>
+      </c>
+      <c r="W9" s="3" t="n">
+        <v>1.479</v>
+      </c>
+      <c r="X9" s="3" t="n">
+        <v>0.297</v>
+      </c>
+      <c r="Y9" s="3" t="n">
+        <v>0.246</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -10759,6 +13506,21 @@
       <c r="T10" s="3" t="n">
         <v>0.015</v>
       </c>
+      <c r="U10" s="3" t="n">
+        <v>1.295</v>
+      </c>
+      <c r="V10" s="3" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="W10" s="3" t="n">
+        <v>1.357</v>
+      </c>
+      <c r="X10" s="3" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="Y10" s="3" t="n">
+        <v>0.199</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -10820,6 +13582,21 @@
       </c>
       <c r="T11" s="3" t="n">
         <v>0.012</v>
+      </c>
+      <c r="U11" s="3" t="n">
+        <v>1.196</v>
+      </c>
+      <c r="V11" s="3" t="n">
+        <v>0.988</v>
+      </c>
+      <c r="W11" s="3" t="n">
+        <v>1.253</v>
+      </c>
+      <c r="X11" s="3" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="Y11" s="3" t="n">
+        <v>0.165</v>
       </c>
     </row>
   </sheetData>
@@ -13217,13 +15994,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13254,6 +16032,11 @@
           <t>+ Scope11</t>
         </is>
       </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>+ Scope8</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -13268,6 +16051,9 @@
       <c r="D3" s="3" t="n">
         <v>1.275</v>
       </c>
+      <c r="E3" s="3" t="n">
+        <v>1.165</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -13282,6 +16068,9 @@
       <c r="D4" s="3" t="n">
         <v>1.211</v>
       </c>
+      <c r="E4" s="3" t="n">
+        <v>1.115</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -13296,6 +16085,9 @@
       <c r="D5" s="3" t="n">
         <v>1.157</v>
       </c>
+      <c r="E5" s="3" t="n">
+        <v>1.074</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -13310,6 +16102,9 @@
       <c r="D6" s="3" t="n">
         <v>1.111</v>
       </c>
+      <c r="E6" s="3" t="n">
+        <v>1.039</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -13324,6 +16119,9 @@
       <c r="D7" s="3" t="n">
         <v>1.104</v>
       </c>
+      <c r="E7" s="3" t="n">
+        <v>1.153</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -13338,6 +16136,9 @@
       <c r="D8" s="3" t="n">
         <v>1.14</v>
       </c>
+      <c r="E8" s="3" t="n">
+        <v>1.167</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -13352,6 +16153,9 @@
       <c r="D9" s="3" t="n">
         <v>1.123</v>
       </c>
+      <c r="E9" s="3" t="n">
+        <v>1.141</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -13366,6 +16170,9 @@
       <c r="D10" s="3" t="n">
         <v>1.033</v>
       </c>
+      <c r="E10" s="3" t="n">
+        <v>1.089</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -13380,6 +16187,9 @@
       <c r="D11" s="3" t="n">
         <v>0.9360000000000001</v>
       </c>
+      <c r="E11" s="3" t="n">
+        <v>0.983</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -13394,6 +16204,9 @@
       <c r="D12" s="3" t="n">
         <v>0.84</v>
       </c>
+      <c r="E12" s="3" t="n">
+        <v>0.869</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -13408,10 +16221,13 @@
       <c r="D13" s="3" t="n">
         <v>0.76</v>
       </c>
+      <c r="E13" s="3" t="n">
+        <v>0.776</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>